<commit_message>
feat: add source links to all W17 promotions
- Jins slides: 6 article links from jins.com/tw/news
- 眼鏡市場 slides: 4 article links from meganeichiba.com.tw/news
- Klassic slides: 2 links from klassicglobal.com
- 母親節總覽表: all 5 promotions linked
- Excel 資料來源URL column: rows 26-34 filled

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/競爭對手追蹤.xlsx
+++ b/競爭對手追蹤.xlsx
@@ -2251,7 +2251,7 @@
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>https://www.jins.com/tw/news/news-69ca36cf22069</t>
+          <t>https://www.jins.com/tw/news/news-69ca367f3b199</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>https://www.jins.com/tw/news</t>
+          <t>https://www.jins.com/tw/news/news-69ca36fe489e3</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="M32" s="17" t="inlineStr">
         <is>
-          <t>https://www.jins.com/tw/news</t>
+          <t>https://www.jins.com/tw/news/news-69ca377bd183c</t>
         </is>
       </c>
     </row>
@@ -2658,39 +2658,44 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>2026/04/13</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>Jins</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="17" t="inlineStr">
         <is>
           <t>品牌活動</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="17" t="inlineStr">
         <is>
           <t>動物平權《野餐我PET你》滾草皮音樂市集</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="17" t="inlineStr">
         <is>
           <t>4/18-4/19</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="17" t="inlineStr">
         <is>
           <t>台北華山大草原</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="17" t="inlineStr">
         <is>
           <t>品牌公關活動，非直接促銷但提升品牌好感度</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>https://www.jins.com/tw/news/news-69d4a2dd8376b</t>
         </is>
       </c>
     </row>

</xml_diff>